<commit_message>
linked wells updates re: w061 to mw and w427 to IO1
</commit_message>
<xml_diff>
--- a/data/input_template_2026.xlsx
+++ b/data/input_template_2026.xlsx
@@ -733,7 +733,6 @@
       <c r="I2" t="b">
         <v>1</v>
       </c>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -777,7 +776,6 @@
       <c r="I3" t="b">
         <v>1</v>
       </c>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -821,7 +819,6 @@
       <c r="I4" t="b">
         <v>1</v>
       </c>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -865,7 +862,6 @@
       <c r="I5" t="b">
         <v>0</v>
       </c>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -909,7 +905,6 @@
       <c r="I6" t="b">
         <v>0</v>
       </c>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -953,7 +948,6 @@
       <c r="I7" t="b">
         <v>0</v>
       </c>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -997,7 +991,6 @@
       <c r="I8" t="b">
         <v>1</v>
       </c>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1041,7 +1034,6 @@
       <c r="I9" t="b">
         <v>1</v>
       </c>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1085,7 +1077,6 @@
       <c r="I10" t="b">
         <v>1</v>
       </c>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1129,7 +1120,6 @@
       <c r="I11" t="b">
         <v>1</v>
       </c>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1173,7 +1163,6 @@
       <c r="I12" t="b">
         <v>1</v>
       </c>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1217,7 +1206,6 @@
       <c r="I13" t="b">
         <v>1</v>
       </c>
-      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1261,7 +1249,6 @@
       <c r="I14" t="b">
         <v>1</v>
       </c>
-      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1305,7 +1292,6 @@
       <c r="I15" t="b">
         <v>1</v>
       </c>
-      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1349,7 +1335,6 @@
       <c r="I16" t="b">
         <v>0</v>
       </c>
-      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1393,7 +1378,6 @@
       <c r="I17" t="b">
         <v>1</v>
       </c>
-      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1437,7 +1421,6 @@
       <c r="I18" t="b">
         <v>1</v>
       </c>
-      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1481,7 +1464,6 @@
       <c r="I19" t="b">
         <v>1</v>
       </c>
-      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1525,7 +1507,6 @@
       <c r="I20" t="b">
         <v>1</v>
       </c>
-      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1569,7 +1550,6 @@
       <c r="I21" t="b">
         <v>1</v>
       </c>
-      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1613,7 +1593,6 @@
       <c r="I22" t="b">
         <v>1</v>
       </c>
-      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1657,7 +1636,6 @@
       <c r="I23" t="b">
         <v>0</v>
       </c>
-      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1701,7 +1679,6 @@
       <c r="I24" t="b">
         <v>0</v>
       </c>
-      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1745,7 +1722,6 @@
       <c r="I25" t="b">
         <v>1</v>
       </c>
-      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1789,7 +1765,6 @@
       <c r="I26" t="b">
         <v>1</v>
       </c>
-      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1833,7 +1808,6 @@
       <c r="I27" t="b">
         <v>1</v>
       </c>
-      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1877,7 +1851,6 @@
       <c r="I28" t="b">
         <v>1</v>
       </c>
-      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1921,7 +1894,6 @@
       <c r="I29" t="b">
         <v>1</v>
       </c>
-      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1965,7 +1937,6 @@
       <c r="I30" t="b">
         <v>0</v>
       </c>
-      <c r="J30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2512,7 +2483,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>W061</t>
+          <t>W427</t>
         </is>
       </c>
     </row>
@@ -2818,7 +2789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2841,11 +2812,6 @@
       <c r="C1" s="1" t="inlineStr">
         <is>
           <t>status</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>status_code</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
IO1/BP2/LW2 linked wells per Tim: W061 + W243 as monitoring wells, W229 renamed V229, W426 added to LW2
- linked_wells: LW2 W243 -> W426 (irrigation-season exempt), drop BP2 W229; optional note column (W427, W426)
- historic_linked_wells: add BP2 W229 (display V229) and LW2 W243 alongside IO1 W061, with display_id/well_status/note
- site cards: table-driven linked-well notes and 'monitoring wells (formerly linked)' rows
- pumping plots: historic series kept; W229 series labelled 'V229 (formerly W229)' (join stays on W229)
- generate_site_maps.R: linked wells from canonical workbook, historic wells drawn as monitoring wells,
  wells without coordinates listed in caption (W426), PUMPING_MAP_SITES subset
- regenerate IO1/BP2/LW2 maps and re-render index/TA-BG
</commit_message>
<xml_diff>
--- a/data/input_template_2026.xlsx
+++ b/data/input_template_2026.xlsx
@@ -161,11 +161,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_linked_wells" displayName="tbl_linked_wells" ref="A1:B61" headerRowCount="1">
-  <autoFilter ref="A1:B61"/>
-  <tableColumns count="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_linked_wells" displayName="tbl_linked_wells" ref="A1:C60" headerRowCount="1">
+  <autoFilter ref="A1:C60"/>
+  <tableColumns count="3">
     <tableColumn id="1" name="site"/>
     <tableColumn id="2" name="well_id"/>
+    <tableColumn id="3" name="note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -609,7 +610,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Static mapping from monitoring site to production wells. Review only when linked well assignments change.</t>
+          <t>Static mapping from monitoring site to production wells. Review only when linked well assignments change. Optional: note (shown on the site card, e.g. exempt status / replacement).</t>
         </is>
       </c>
     </row>
@@ -1952,11 +1953,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1970,6 +1972,11 @@
           <t>well_id</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2051,7 +2058,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>W243</t>
+          <t>W426</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Irrigation-season exempt; replaced W243 (now a monitoring well).</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2207,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>W229</t>
+          <t>W374</t>
         </is>
       </c>
     </row>
@@ -2207,19 +2219,19 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>W374</t>
+          <t>W375</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BP2</t>
+          <t>BP3</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>W375</t>
+          <t>W222</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2243,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>W222</t>
+          <t>W223</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2255,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>W223</t>
+          <t>W231</t>
         </is>
       </c>
     </row>
@@ -2255,31 +2267,31 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>W231</t>
+          <t>W232</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BP3</t>
+          <t>BP4</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>W232</t>
+          <t>W331</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BP4</t>
+          <t>TA3</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>W331</t>
+          <t>W106</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2303,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>W106</t>
+          <t>W110</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2315,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>W110</t>
+          <t>W111</t>
         </is>
       </c>
     </row>
@@ -2315,19 +2327,19 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>W111</t>
+          <t>W114</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TA3</t>
+          <t>TA4</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>W114</t>
+          <t>W342</t>
         </is>
       </c>
     </row>
@@ -2339,31 +2351,31 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>W342</t>
+          <t>W347</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TA4</t>
+          <t>TA5</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>W347</t>
+          <t>W349</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TA5</t>
+          <t>TA6</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>W349</t>
+          <t>W109</t>
         </is>
       </c>
     </row>
@@ -2375,43 +2387,43 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>W109</t>
+          <t>W370</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TA6</t>
+          <t>TS1</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>W370</t>
+          <t>W159</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TS1</t>
+          <t>TS2</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>W159</t>
+          <t>W155</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TS2</t>
+          <t>TS3</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>W155</t>
+          <t>W103</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2435,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>W103</t>
+          <t>W104</t>
         </is>
       </c>
     </row>
@@ -2435,19 +2447,19 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>W104</t>
+          <t>W382</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TS3</t>
+          <t>TS4</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>W382</t>
+          <t>W380</t>
         </is>
       </c>
     </row>
@@ -2459,19 +2471,24 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>W380</t>
+          <t>W381</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TS4</t>
+          <t>IO1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>W381</t>
+          <t>W427</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Irrigation-season exempt; replaced W061 (now a monitoring well).</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2500,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>W427</t>
+          <t>W391</t>
         </is>
       </c>
     </row>
@@ -2495,31 +2512,31 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>W391</t>
+          <t>W400</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IO1</t>
+          <t>IO2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>W400</t>
+          <t>W063</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IO2</t>
+          <t>SS1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>W063</t>
+          <t>W069</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2548,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>W069</t>
+          <t>W392</t>
         </is>
       </c>
     </row>
@@ -2543,19 +2560,19 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>W392</t>
+          <t>W393</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SS1</t>
+          <t>SS2</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>W393</t>
+          <t>W074</t>
         </is>
       </c>
     </row>
@@ -2567,7 +2584,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>W074</t>
+          <t>W394</t>
         </is>
       </c>
     </row>
@@ -2579,19 +2596,19 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>W394</t>
+          <t>W395</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SS2</t>
+          <t>SS3</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>W395</t>
+          <t>W092</t>
         </is>
       </c>
     </row>
@@ -2603,19 +2620,19 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>W092</t>
+          <t>W396</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SS3</t>
+          <t>SS4</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>W396</t>
+          <t>W075</t>
         </is>
       </c>
     </row>
@@ -2627,19 +2644,19 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>W075</t>
+          <t>W345</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SS4</t>
+          <t>BG2</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>W345</t>
+          <t>W076</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2668,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>W076</t>
+          <t>W403</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2680,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>W403</t>
+          <t>W343</t>
         </is>
       </c>
     </row>
@@ -2674,18 +2691,6 @@
         </is>
       </c>
       <c r="B60" t="inlineStr">
-        <is>
-          <t>W343</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>BG2</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
         <is>
           <t>W348</t>
         </is>

</xml_diff>